<commit_message>
Descripción de los cambios
</commit_message>
<xml_diff>
--- a/historico_descuentos.xlsx
+++ b/historico_descuentos.xlsx
@@ -4129,7 +4129,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z19"/>
+  <dimension ref="A1:Z22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4895,9 +4895,124 @@
         <v>Zona 2_x000d_</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Septiembre 2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>AMINA MAHMAD ABDEL (COMERCIAL ZITAWI MAHMAD F.P.)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>FACTF/2026/11712</v>
+      </c>
+      <c r="D20" t="str">
+        <v>OEG-4BTE</v>
+      </c>
+      <c r="E20" t="str">
+        <v>1</v>
+      </c>
+      <c r="F20" t="str">
+        <v>115,00</v>
+      </c>
+      <c r="G20" t="str">
+        <v>103,50</v>
+      </c>
+      <c r="H20" t="str">
+        <v>11,50</v>
+      </c>
+      <c r="I20" t="str">
+        <v>11,50</v>
+      </c>
+      <c r="J20" t="str">
+        <v>10%</v>
+      </c>
+      <c r="K20" t="str">
+        <v xml:space="preserve">Critico </v>
+      </c>
+      <c r="L20" t="str">
+        <v>Zona 3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Septiembre 2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>DISTRIBUIDORA AMADO 2020, C.A.</v>
+      </c>
+      <c r="C21" t="str">
+        <v>FACTF/2026/09790</v>
+      </c>
+      <c r="D21" t="str">
+        <v>OCH-198W</v>
+      </c>
+      <c r="E21" t="str">
+        <v>1</v>
+      </c>
+      <c r="F21" t="str">
+        <v>220,00</v>
+      </c>
+      <c r="G21" t="str">
+        <v>204,60</v>
+      </c>
+      <c r="H21" t="str">
+        <v>15,40</v>
+      </c>
+      <c r="I21" t="str">
+        <v>15,40</v>
+      </c>
+      <c r="J21" t="str">
+        <v>7%</v>
+      </c>
+      <c r="K21" t="str">
+        <v xml:space="preserve">Critico </v>
+      </c>
+      <c r="L21" t="str">
+        <v>Zona 1_x000d_</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>Septiembre 2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>INVERSIONES CASANOVA ELECTRONIC 2009, C.A</v>
+      </c>
+      <c r="C22" t="str">
+        <v>FACTF/2026/09108</v>
+      </c>
+      <c r="D22" t="str">
+        <v>OCH-198W</v>
+      </c>
+      <c r="E22" t="str">
+        <v>1</v>
+      </c>
+      <c r="F22" t="str">
+        <v>220,00</v>
+      </c>
+      <c r="G22" t="str">
+        <v>204,60</v>
+      </c>
+      <c r="H22" t="str">
+        <v>15,40</v>
+      </c>
+      <c r="I22" t="str">
+        <v>15,40</v>
+      </c>
+      <c r="J22" t="str">
+        <v>7%</v>
+      </c>
+      <c r="K22" t="str">
+        <v xml:space="preserve">Critico </v>
+      </c>
+      <c r="L22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Zona 1
+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>